<commit_message>
added a feature selection pipeline
</commit_message>
<xml_diff>
--- a/Children_EDA_Summary.xlsx
+++ b/Children_EDA_Summary.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/naghamdaood/Projects/TATOO/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D740CF-3F51-8348-A8FD-EDDF1FA67CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="16920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demographics" sheetId="1" r:id="rId1"/>
@@ -18,7 +24,7 @@
     <sheet name="T13" sheetId="9" r:id="rId9"/>
     <sheet name="T20" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -922,8 +928,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -975,8 +981,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -986,13 +995,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1030,7 +1047,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1064,6 +1081,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1098,9 +1116,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1273,11 +1292,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1297,7 +1324,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1317,7 +1344,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1337,7 +1364,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1363,29 +1390,29 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1417,12 +1444,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>270</v>
       </c>
@@ -1439,7 +1466,7 @@
         <v>5.85</v>
       </c>
       <c r="F4">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G4">
         <v>3.75</v>
@@ -1454,7 +1481,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>271</v>
       </c>
@@ -1486,7 +1513,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>272</v>
       </c>
@@ -1497,7 +1524,7 @@
         <v>97.5</v>
       </c>
       <c r="D6">
-        <v>99.65000000000001</v>
+        <v>99.65</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -1518,7 +1545,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>273</v>
       </c>
@@ -1529,7 +1556,7 @@
         <v>1.5</v>
       </c>
       <c r="D7">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1550,7 +1577,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>274</v>
       </c>
@@ -1582,7 +1609,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>275</v>
       </c>
@@ -1614,12 +1641,12 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>276</v>
       </c>
       <c r="B10">
-        <v>2.22</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="C10">
         <v>1.33</v>
@@ -1646,7 +1673,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>277</v>
       </c>
@@ -1654,7 +1681,7 @@
         <v>13.13</v>
       </c>
       <c r="C11">
-        <v>9.859999999999999</v>
+        <v>9.86</v>
       </c>
       <c r="D11">
         <v>9.84</v>
@@ -1678,7 +1705,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>278</v>
       </c>
@@ -1710,7 +1737,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>279</v>
       </c>
@@ -1753,29 +1780,40 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="11.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1807,12 +1845,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1820,7 +1858,7 @@
         <v>23.41</v>
       </c>
       <c r="C4">
-        <v>20.26</v>
+        <v>20.260000000000002</v>
       </c>
       <c r="D4">
         <v>25.83</v>
@@ -1844,7 +1882,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
@@ -1876,7 +1914,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -1908,7 +1946,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -1916,10 +1954,10 @@
         <v>0.27</v>
       </c>
       <c r="C7">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D7">
-        <v>32.02</v>
+        <v>32.020000000000003</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1940,7 +1978,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -1948,10 +1986,10 @@
         <v>97.77</v>
       </c>
       <c r="C8">
-        <v>99.06999999999999</v>
+        <v>99.07</v>
       </c>
       <c r="D8">
-        <v>66.01000000000001</v>
+        <v>66.010000000000005</v>
       </c>
       <c r="E8">
         <v>100</v>
@@ -1972,7 +2010,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>27</v>
       </c>
@@ -1983,7 +2021,7 @@
         <v>0.86</v>
       </c>
       <c r="D9">
-        <v>2.07</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -2004,12 +2042,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B10">
-        <v>2.53</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="C10">
         <v>1.44</v>
@@ -2021,7 +2059,7 @@
         <v>2.04</v>
       </c>
       <c r="F10">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="G10">
         <v>2.12</v>
@@ -2047,29 +2085,29 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2101,12 +2139,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>50</v>
       </c>
@@ -2138,7 +2176,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>51</v>
       </c>
@@ -2152,13 +2190,13 @@
         <v>8.66</v>
       </c>
       <c r="E5">
-        <v>9.300000000000001</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="F5">
         <v>8.1</v>
       </c>
       <c r="G5">
-        <v>8.449999999999999</v>
+        <v>8.4499999999999993</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
@@ -2170,7 +2208,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -2178,7 +2216,7 @@
         <v>12.93</v>
       </c>
       <c r="C6">
-        <v>9.859999999999999</v>
+        <v>9.86</v>
       </c>
       <c r="D6">
         <v>8.93</v>
@@ -2202,7 +2240,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>53</v>
       </c>
@@ -2234,7 +2272,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>54</v>
       </c>
@@ -2254,7 +2292,7 @@
         <v>0.5</v>
       </c>
       <c r="G8">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="H8" t="s">
         <v>63</v>
@@ -2266,7 +2304,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>55</v>
       </c>
@@ -2298,7 +2336,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
@@ -2306,7 +2344,7 @@
         <v>18.47</v>
       </c>
       <c r="C10">
-        <v>8.640000000000001</v>
+        <v>8.64</v>
       </c>
       <c r="D10">
         <v>10.25</v>
@@ -2330,7 +2368,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>57</v>
       </c>
@@ -2338,7 +2376,7 @@
         <v>80.67</v>
       </c>
       <c r="C11">
-        <v>89.56999999999999</v>
+        <v>89.57</v>
       </c>
       <c r="D11">
         <v>89.88</v>
@@ -2362,7 +2400,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>58</v>
       </c>
@@ -2394,7 +2432,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>59</v>
       </c>
@@ -2437,29 +2475,29 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2491,23 +2529,23 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B4">
-        <v>8.699999999999999</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="C4">
         <v>10</v>
       </c>
       <c r="D4">
-        <v>10.05</v>
+        <v>10.050000000000001</v>
       </c>
       <c r="E4">
         <v>10</v>
@@ -2528,7 +2566,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>88</v>
       </c>
@@ -2542,7 +2580,7 @@
         <v>10.94</v>
       </c>
       <c r="E5">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="F5">
         <v>7.6</v>
@@ -2560,7 +2598,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>89</v>
       </c>
@@ -2592,7 +2630,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>90</v>
       </c>
@@ -2624,7 +2662,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>91</v>
       </c>
@@ -2656,7 +2694,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>92</v>
       </c>
@@ -2688,7 +2726,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>93</v>
       </c>
@@ -2720,7 +2758,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>94</v>
       </c>
@@ -2728,7 +2766,7 @@
         <v>97.33</v>
       </c>
       <c r="C11">
-        <v>99.29000000000001</v>
+        <v>99.29</v>
       </c>
       <c r="D11">
         <v>97.03</v>
@@ -2752,7 +2790,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>95</v>
       </c>
@@ -2784,7 +2822,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>96</v>
       </c>
@@ -2827,29 +2865,32 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2881,12 +2922,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>122</v>
       </c>
@@ -2918,7 +2959,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
@@ -2950,7 +2991,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>124</v>
       </c>
@@ -2982,7 +3023,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>125</v>
       </c>
@@ -3014,7 +3055,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>126</v>
       </c>
@@ -3046,7 +3087,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>127</v>
       </c>
@@ -3078,7 +3119,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>128</v>
       </c>
@@ -3110,7 +3151,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>129</v>
       </c>
@@ -3142,7 +3183,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>130</v>
       </c>
@@ -3174,7 +3215,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>131</v>
       </c>
@@ -3217,29 +3258,35 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3271,12 +3318,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>149</v>
       </c>
@@ -3308,7 +3355,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>150</v>
       </c>
@@ -3340,7 +3387,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>151</v>
       </c>
@@ -3372,7 +3419,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>152</v>
       </c>
@@ -3404,7 +3451,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>153</v>
       </c>
@@ -3436,7 +3483,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>154</v>
       </c>
@@ -3447,7 +3494,7 @@
         <v>132</v>
       </c>
       <c r="D9">
-        <v>95.59999999999999</v>
+        <v>95.6</v>
       </c>
       <c r="E9" t="s">
         <v>132</v>
@@ -3468,7 +3515,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>155</v>
       </c>
@@ -3500,7 +3547,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>156</v>
       </c>
@@ -3532,7 +3579,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>157</v>
       </c>
@@ -3564,7 +3611,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>158</v>
       </c>
@@ -3575,7 +3622,7 @@
         <v>132</v>
       </c>
       <c r="D13">
-        <v>33.95</v>
+        <v>33.950000000000003</v>
       </c>
       <c r="E13" t="s">
         <v>132</v>
@@ -3596,7 +3643,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>159</v>
       </c>
@@ -3628,7 +3675,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>160</v>
       </c>
@@ -3660,7 +3707,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>161</v>
       </c>
@@ -3692,7 +3739,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>162</v>
       </c>
@@ -3724,7 +3771,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>163</v>
       </c>
@@ -3744,7 +3791,7 @@
         <v>132</v>
       </c>
       <c r="G18">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="H18" t="s">
         <v>132</v>
@@ -3756,7 +3803,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>164</v>
       </c>
@@ -3788,7 +3835,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>165</v>
       </c>
@@ -3820,7 +3867,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>166</v>
       </c>
@@ -3852,7 +3899,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>167</v>
       </c>
@@ -3884,7 +3931,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>168</v>
       </c>
@@ -3916,7 +3963,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>169</v>
       </c>
@@ -3948,7 +3995,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>170</v>
       </c>
@@ -3980,7 +4027,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>171</v>
       </c>
@@ -4012,7 +4059,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>172</v>
       </c>
@@ -4055,29 +4102,29 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4109,12 +4156,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>190</v>
       </c>
@@ -4146,7 +4193,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>191</v>
       </c>
@@ -4178,7 +4225,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>192</v>
       </c>
@@ -4186,10 +4233,10 @@
         <v>132</v>
       </c>
       <c r="C6">
-        <v>9.789999999999999</v>
+        <v>9.7899999999999991</v>
       </c>
       <c r="D6">
-        <v>10.05</v>
+        <v>10.050000000000001</v>
       </c>
       <c r="E6" t="s">
         <v>132</v>
@@ -4210,7 +4257,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>193</v>
       </c>
@@ -4242,7 +4289,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>194</v>
       </c>
@@ -4253,7 +4300,7 @@
         <v>55.88</v>
       </c>
       <c r="D8">
-        <v>71.48999999999999</v>
+        <v>71.489999999999995</v>
       </c>
       <c r="E8" t="s">
         <v>132</v>
@@ -4274,7 +4321,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>195</v>
       </c>
@@ -4306,7 +4353,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>196</v>
       </c>
@@ -4338,7 +4385,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>197</v>
       </c>
@@ -4370,7 +4417,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>198</v>
       </c>
@@ -4402,7 +4449,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>199</v>
       </c>
@@ -4445,29 +4492,32 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4499,12 +4549,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>216</v>
       </c>
@@ -4536,7 +4586,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>217</v>
       </c>
@@ -4568,12 +4618,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>218</v>
       </c>
       <c r="B6">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -4600,7 +4650,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>219</v>
       </c>
@@ -4632,7 +4682,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>220</v>
       </c>
@@ -4664,12 +4714,12 @@
         <v>239</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>221</v>
       </c>
       <c r="B9">
-        <v>9.470000000000001</v>
+        <v>9.4700000000000006</v>
       </c>
       <c r="C9">
         <v>2.14</v>
@@ -4696,7 +4746,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>222</v>
       </c>
@@ -4713,7 +4763,7 @@
         <v>18.5</v>
       </c>
       <c r="F10">
-        <v>8.550000000000001</v>
+        <v>8.5500000000000007</v>
       </c>
       <c r="G10">
         <v>13.95</v>
@@ -4728,7 +4778,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>223</v>
       </c>
@@ -4771,29 +4821,32 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4825,12 +4878,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>243</v>
       </c>
@@ -4862,7 +4915,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>244</v>
       </c>
@@ -4894,7 +4947,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>245</v>
       </c>
@@ -4926,7 +4979,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>246</v>
       </c>
@@ -4937,7 +4990,7 @@
         <v>15.86</v>
       </c>
       <c r="D7">
-        <v>17.51</v>
+        <v>17.510000000000002</v>
       </c>
       <c r="E7">
         <v>21.5</v>
@@ -4958,7 +5011,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>247</v>
       </c>
@@ -4990,15 +5043,15 @@
         <v>266</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>248</v>
       </c>
       <c r="B9">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="C9">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D9">
         <v>0.96</v>
@@ -5022,7 +5075,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>249</v>
       </c>
@@ -5054,7 +5107,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>250</v>
       </c>
@@ -5062,10 +5115,10 @@
         <v>12.73</v>
       </c>
       <c r="C11">
-        <v>9.869999999999999</v>
+        <v>9.8699999999999992</v>
       </c>
       <c r="D11">
-        <v>9.869999999999999</v>
+        <v>9.8699999999999992</v>
       </c>
       <c r="E11">
         <v>11.45</v>
@@ -5074,7 +5127,7 @@
         <v>7.3</v>
       </c>
       <c r="G11">
-        <v>8.449999999999999</v>
+        <v>8.4499999999999993</v>
       </c>
       <c r="H11" t="s">
         <v>257</v>

</xml_diff>